<commit_message>
Add Muse and Instinct impact analysis on direct marketplace traffic
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Assistants_Marketplace_Traffic_Uber_DoorDash_Airbnb.xlsx
+++ b/AI_Assistants_Marketplace_Traffic_Uber_DoorDash_Airbnb.xlsx
@@ -13,7 +13,8 @@
     <sheet name="DoorDash" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Airbnb" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Comparison" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Muse &amp; Instinct Impact" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +53,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
     </font>
     <font>
       <color rgb="000563C1"/>
@@ -102,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,10 +128,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -492,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -588,22 +596,34 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>How to read this file</t>
+          <t>Key takeaway 6</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>'Industry Traffic Data' holds cross-industry quantitative benchmarks. The Uber, DoorDash, and Airbnb sheets hold company-specific findings with dates and sources. 'Comparison' is a side-by-side matrix. 'Sources' lists every reference with URLs.</t>
+          <t>A new class of autonomous personal agents - Meta's Muse (launched Sep 8, 2026) and startup Instinct - raises the stakes beyond ChatGPT-style integrations. These agents open their own browser, fill forms, and pay with Stripe Link virtual cards, so they can transact on Uber, DoorDash, or Airbnb WITHOUT a partnership and without the human ever visiting the marketplace's app or site. That threatens direct traffic, ad impressions, and membership loops - though volumes are negligible today. See the 'Muse &amp; Instinct Impact' sheet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>How to read this file</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>'Industry Traffic Data' holds cross-industry quantitative benchmarks. The Uber, DoorDash, and Airbnb sheets hold company-specific findings with dates and sources. 'Comparison' is a side-by-side matrix. 'Muse &amp; Instinct Impact' covers the new autonomous personal agents and their potential effect on direct traffic. 'Sources' lists every reference with URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Caveat</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>None of the three companies has disclosed the absolute volume or revenue share of AI-assistant-referred traffic. Directional claims (e.g., 'converts better than Google') come from executives without underlying figures; industry-level percentages come from Adobe Analytics and Similarweb panels, not company filings.</t>
         </is>
@@ -1885,10 +1905,393 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Muse (Meta) &amp; Instinct: Potential Impact on Direct Marketplace Traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous personal agents that act on websites and pay on the user's behalf - a different threat model than ChatGPT-style in-chat apps. Compiled September 15, 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Agent profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Muse (Meta)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Instinct (Spear Street Technology)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Why it matters for marketplace traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>What it is / status</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Personal AI agent from Meta Superintelligence Labs (internally 'Hatch'). Launched US-only Sep 8, 2026 on iOS, Android, muse.ai, and inside WhatsApp; AI glasses support coming. Free tier plus reported $20/$100 per month subscriptions.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Consumer AI agent that works over ordinary SMS text messages and phone calls - no app install. Private access with a waitlist; no published pricing. Raised ~$250-350M (reports differ) at a $2.5B valuation in late Aug 2026.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Both are 'do-er' agents, not chatbots: the promise is that the user never opens the marketplace app at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>How it executes tasks</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Runs on a dedicated per-user 'Muse Secure VM' with its own browser; opens websites, fills out forms, negotiates, books travel, sells items. Launch connectors: Instagram, Facebook, Gmail, Google Calendar, Ticketmaster, OpenTable, Spotify, Apple Health, Plaid, Shopify. For everything else, it 'can use the website directly.'</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Acts on any web page on the user's behalf; supports 1Password credential sharing so it can log into existing accounts. Ships features at high velocity; launched an agent-to-agent protocol where one user's agent coordinates plans with a friend's agent over SMS.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Neither agent needs the marketplace's permission or a formal integration: browser automation plus stored credentials reach any site, including Uber, DoorDash, and Airbnb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Checks out with Stripe Link's wallet for agents: instant checkout at 1M+ Link-accepting businesses; elsewhere a single-use virtual card scoped to the approved purchase. First agent covered by Link purchase protections (returns, price drops, damaged items); user approves each total in chat. Shop Pay support coming.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Also uses Stripe Link's agent wallet for payments (Stripe names Instinct and Grok Bot as earlier Link agent-wallet users), plus 1Password for logins.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Agent-native payment rails remove the last reason to hand off to the marketplace's own app - unlike ChatGPT's Uber/DoorDash apps, where checkout still happens in-app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Distribution &amp; early traction</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>WhatsApp integration at launch; Meta says it will rerun the Threads playbook (0 to 500M MAU via Instagram) for AI apps. ~4.3M US iOS downloads on day one, hitting No. 2 on iOS, but weak Android traction (No. 338 in Productivity) and launch analyses called the numbers underwhelming.</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Growth constrained by invite/waitlist and compute; SMS interface means zero-install adoption once open. Hype-driven demand; described as 'the hottest startup in the category.'</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Meta's billions-scale distribution is the main reason to take agent-mediated traffic seriously despite tiny current volumes; Instinct shows the interface can be as thin as a text thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Trust &amp; controversy</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Reuters reported internal tests showed the agent stalling and mismanaging access to sensitive data; Meta counters with VM isolation, audit trails, approval prompts, and no visibility into passwords or card numbers.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Criticized for a 'perpetual and irrevocable' data license in its terms and for sending an email on a user's behalf without asking.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Trust failures slow consumer adoption of agent-mediated transactions - currently the biggest brake on any traffic impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Potential impact channels on direct marketplace traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Impact channel</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Mechanism</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Potential effect on direct traffic</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Relative exposure: Uber / DoorDash / Airbnb</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Substitution of human visits</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>User messages Muse (in WhatsApp) or texts Instinct - 'get me a ride to the airport,' 'order dinner for four,' 'book a place in Austin' - and the agent completes the task in its own browser session.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Direct traffic (app opens, typed-URL and organic sessions) is replaced by agent sessions. The human never sees the marketplace's home feed, promotions, or search results, even though the transaction still happens on the platform.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Uber: lower near-term risk - real-time pickup logistics and location favor the native app. DoorDash: high - meal ordering is a routine, delegable task. Airbnb: medium - high-consideration stays still pull humans in, but agents can shortlist and even book.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Loss of advertising &amp; sponsored-listing impressions</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Marketplace ad businesses (DoorDash ads, Uber's advertising arm, Airbnb's planned sponsored listings in AI search) monetize human eyeballs on search/browse surfaces. An agent parsing a page doesn't 'view' ads and may ignore sponsored placement entirely.</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Even traffic that still technically lands on the marketplace loses monetizable impressions; ad load could become a reason agents route around the consumer front-end to cleaner data sources.</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>DoorDash most exposed (ads are a core profit stream); Uber increasingly exposed as its ads business grows; Airbnb least exposed today but its planned AI-search sponsorships assume human viewers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Erosion of membership &amp; cross-sell loops</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Uber One and DashPass economics, and Uber's cross-platform strategy (members spend ~3x more), depend on humans inside the app seeing upsells, bundles, and other verticals.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>If agents execute single transactions on command, marketplaces lose the browsing moments that drive membership sign-ups and cross-category discovery - flattening lifetime value even if order counts hold.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Uber and DoorDash highly exposed (membership-driven models); Airbnb less so (no subscription program), though its new social and services features assume in-app time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Attribution &amp; analytics distortion</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Muse's per-user VM browser and Link's single-use virtual cards make agent sessions look like anonymous direct/bot traffic; Instinct logging in with a user's stored 1Password credentials looks like the human returning.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Reported 'direct traffic' becomes unreliable in both directions: genuine agent-mediated demand may be blocked as bot traffic, while measured direct sessions overstate human engagement. Marketing mix and conversion models degrade.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>All three roughly equally exposed; whichever builds agent-recognition (verified agent lanes, agent APIs) first will measure - and price - this demand instead of guessing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Demand aggregation via agent-to-agent coordination</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Instinct's agent-to-agent SMS protocol lets one user's agent negotiate weekend plans with a friend's agent; Muse plans goal-level coordination ('plan the trip'), not single tasks.</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Group decisions (where to stay, where to eat, how to get there) could be settled between agents before any marketplace is consulted - the marketplaces receive a fully-formed booking request, with zero upstream discovery traffic to influence.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Airbnb most exposed on trip planning (group stays), DoorDash on group orders and reservations (SevenRooms), Uber on shared rides to coordinated events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Platform conflict: Meta's own marketplace ambitions</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Meta is wiring Muse into Facebook Marketplace (AI listing drafts, auto-replies, full transaction automation with Meta's wallet), and Muse ships with OpenTable - a direct rival to DoorDash-owned SevenRooms - as a launch connector.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Muse is not a neutral router: when Meta monetizes agent-completed transactions, it has an incentive to steer tasks toward partners and its own surfaces, making unpartnered marketplaces' traffic dependent on Meta's choices.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>DoorDash faces the sharpest conflict (reservations); Airbnb competes with any Meta travel ambitions; Uber least conflicted today - no Meta mobility product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Counterweights &amp; moats</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Identity verification (~90% of Airbnb bookers must verify ID - the same barrier that stalled a ChatGPT integration), real-time dynamic pricing (Uber quotes shift within minutes), account requirements, bot detection, and each user approving purchase totals in chat all add friction to fully autonomous transacting.</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>These frictions currently keep agents in an 'assist and hand off' role rather than full substitution - which preserves a (diminished) direct-traffic touchpoint. Marketplaces can also choose to treat verified agents as a channel: official agent APIs would convert the threat into partner-referred volume they can meter.</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Airbnb's ID/trust layer is the strongest natural moat; Uber's real-time logistics second; DoorDash's commodity checkout is the easiest for an agent to complete end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Realistic near-term sizing</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Muse is US-only, days old, with mixed launch traction; Instinct is waitlist-gated. DoorDash already reports external agentic order volume is 'quite low,' and Adobe/Similarweb data show assistant-driven visits are still a small share of marketplace traffic overall.</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Direct-traffic impact in 2026 is negligible-to-small. The structural risk is on the assumptions behind 2027+ plans: ad revenue growth, membership attach rates, and owned-channel marketing all presume humans keep opening the apps.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Watch: Muse WhatsApp usage curves, Instinct's general availability, Stripe Link agent-wallet transaction disclosures, and whether any of the three launches a verified-agent API or blocks agent browsers.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1947,7 +2350,7 @@
           <t>MarTech, Feb 2026</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>https://martech.org/airbnb-says-ai-chatbot-traffic-converts-better-than-google/</t>
         </is>
@@ -1967,7 +2370,7 @@
           <t>Search Engine Land, Feb 2026</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>https://searchengineland.com/airbnb-traffic-ai-chatbots-google-469415</t>
         </is>
@@ -1987,7 +2390,7 @@
           <t>Marketing Week, Feb 2026</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>https://www.marketingweek.com/airbnb-ai-search/</t>
         </is>
@@ -2007,7 +2410,7 @@
           <t>CNBC, Oct 22, 2025</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2025/10/22/airbnb-chatgpt-ai-chesky.html</t>
         </is>
@@ -2027,7 +2430,7 @@
           <t>CNBC, Aug 7, 2026</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/08/07/chesky-airbnb-ai-earnings.html</t>
         </is>
@@ -2047,7 +2450,7 @@
           <t>YouTube, Jan 14, 2026</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7LIPCIhi5aY</t>
         </is>
@@ -2067,7 +2470,7 @@
           <t>Uber Help Center, Nov 2025</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>https://help.uber.com/en/riders/article/chatgpt-integration-for-rides?nodeId=afa53c91-a8e0-4306-b18f-9f742bf24252</t>
         </is>
@@ -2087,7 +2490,7 @@
           <t>Developments Today, 2026</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>https://developmentstoday.com/ai-robotics/uber-is-turning-real-time-marketplace-data-into-ai-guidance-for-drivers-and-ride</t>
         </is>
@@ -2107,7 +2510,7 @@
           <t>PYMNTS, 2026</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>https://www.pymnts.com/artificial-intelligence-2/2026/ubers-ai-knows-the-city-before-your-driver-does/</t>
         </is>
@@ -2127,7 +2530,7 @@
           <t>LinkedIn, May 7, 2026</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/posts/openai-for-business_every-day-uber-runs-a-global-real-time-marketplace-activity-7458185079782014976-ROgl</t>
         </is>
@@ -2147,7 +2550,7 @@
           <t>earningscalls.dev, Sep 10, 2026</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>https://earningscalls.dev/transcripts/uber-technologies-inc_uber_earnings_call_transcript_2026-09-10</t>
         </is>
@@ -2167,7 +2570,7 @@
           <t>DoorDash newsroom, Dec 2025</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>https://about.doordash.com/en-us/news/openai</t>
         </is>
@@ -2187,7 +2590,7 @@
           <t>Digital Commerce 360, Dec 19, 2025</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>https://www.digitalcommerce360.com/2025/12/19/doordash-app-openai-chatgpt/</t>
         </is>
@@ -2207,7 +2610,7 @@
           <t>CNBC, Jun 11, 2026</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/06/11/doordash-ai-ordering-automation.html</t>
         </is>
@@ -2227,7 +2630,7 @@
           <t>TechCrunch, Jun 11, 2026</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>https://techcrunch.com/2026/06/11/doordashs-new-ai-chatbot-lets-you-order-with-prompts-and-photos/</t>
         </is>
@@ -2247,7 +2650,7 @@
           <t>PYMNTS, Aug 2026</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>https://www.pymnts.com/news/delivery/2026/doordash-says-agentic-traffic-is-low-but-ai-gains-are-not/</t>
         </is>
@@ -2267,7 +2670,7 @@
           <t>AInvest, 2026</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>https://www.ainvest.com/news/openai-891-million-users-threaten-uber-eats-doordash-invisible-infrastructure-shift-2604/</t>
         </is>
@@ -2287,7 +2690,7 @@
           <t>UBOS, Mar 2026</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>https://ubos.tech/news/openai-unveils-new-chatgpt-app-integrations-with-doordash-spotify-uber-and-more/</t>
         </is>
@@ -2307,7 +2710,7 @@
           <t>Search Engine Land, Jun 2026</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>https://searchengineland.com/ai-referrals-engagement-travel-sites-adobe-480445</t>
         </is>
@@ -2327,7 +2730,7 @@
           <t>The Letter Two, Aug 21, 2026</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>https://thelettertwo.com/2026/08/21/adobe-ai-travel-traffic-visibility-gap-july-2026/</t>
         </is>
@@ -2347,7 +2750,7 @@
           <t>Forbes, Aug 19, 2026</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>https://www.forbes.com/sites/joanverdon/2026/08/19/ai-is-becoming-a-travelers-best-friend-driving-engagement-and-bookings/</t>
         </is>
@@ -2367,7 +2770,7 @@
           <t>Similarweb, 2026</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>https://aisearch.similarweb.com/blog/ai-referral-traffic-by-industry/</t>
         </is>
@@ -2387,9 +2790,189 @@
           <t>Adobe (mirrored PDF), Apr 2026</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>https://www.defimode.org/wp-content/uploads/2026/04/4226ac98-e5cc-4916-88de-bedc1dd1d584.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Introducing Muse: The World's First Personal AI Agent Built for Everyone</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Meta Newsroom, Sep 8, 2026</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>https://about.fb.com/news/2026/09/introducing-muse-personal-ai-agent/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Meta Releases Muse, a Personal AI Agent With Privacy 'Built Into It'</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>WIRED, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wired.com/story/meta-releases-muse-a-personal-ai-agent-with-privacy-built-into-it/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Meta launches AI agent that can access other apps to send emails, make payments</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Reuters, Sep 8, 2026</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/business/meta-launches-ai-agent-that-can-access-other-apps-send-emails-make-payments-2026-09-08/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Meta just launched its most important product since WhatsApp and Instagram: the Muse AI agent</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>UncoverAlpha, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.uncoveralpha.com/p/meta-just-launched-its-most-important</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Stripe helps Muse, Meta's new personal AI agent, shop across the internet with Link</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Stripe Newsroom, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>https://stripe.com/newsroom/news/stripe-helps-meta-muse-shop-with-link</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Meta Muse AI agent: Everything it can do, and everything it's asking for</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>The Creators Index, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>https://thecreatorsindex.com/platform/meta/meta-muse-ai-agent-everything-it-can-do-and-everything-its-asking-for</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Meta Muse AI Agent Launch: Commerce Moves Beyond Search</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Real Internet Sales, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>https://www.realinternetsales.com/meta-muse-ai-agent-launch-agentic-commerce/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Muse vs Instinct: Which AI Assistant Can You Use?</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Legend Memory, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>https://legendmemory.ai/blogs/the-archive/muse-vs-instinct-ai-assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Meta's new AI agent Muse hits No. 2 on iOS, but the launch numbers look grim</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Singularity Moments, Sep 2026</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>https://singularitymoments.com/content/metas-new-ai-agent-muse-hits-no-2-on-ios-but-the-launch-numbers-look-grim/</t>
         </is>
       </c>
     </row>
@@ -2422,6 +3005,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>